<commit_message>
feat(sanguo-A3+ux): 场景系统美术清单 + 四界面拖动滚动(DragScroll) + 首批CC0 BGM入库
- A3: docs/design/scene_system_art_spec.xlsx(6 sheet/69行——塔分阵营5套/地形3主题/FX18/UI中式小改/头像16/音频方向; 用户4决策入PLAN §0)
- 滚动: view/ui/drag_scroll.gd 通用组件(鼠标按住拖动+轻点派发, 真机触摸走引擎原生);
  组卡/创号/图鉴/闯关四界面接入; 组卡卡池与创号头像网格改 ScrollContainer(修48卡/39头像超屏无滚动阻塞bug);
  首版 emulate_touch_from_mouse 路线失败已撤销(project.godot 净零改动)
- BGM: 菜单=Oriental / 战斗=Ninja Theme(OpenGameArt CC0 可商用免署名, 来源许可记 source_notes);
  AudioManager 补清单 loop 生效(ogg/mp3/wav); tests/test_audio_assets.gd 清单一致性守门
- 验收台账 C组(滚动×5)/D组(BGM×2) + 首轮验收反馈记录; .gitignore 加 Office 锁文件
- 客户端单测 358/358

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/config/AudioConfig.xlsx
+++ b/config/AudioConfig.xlsx
@@ -779,7 +779,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>planned</t>
+          <t>imported</t>
         </is>
       </c>
       <c r="H3" s="2" t="b">
@@ -817,12 +817,12 @@
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>中速战斗循环；鼓点清楚但不要过密，给部署、命中和法术音效留空间。</t>
+          <t>三国战斗循环：古筝+笛动作节奏（热血物语向），鼓点中速给部署/命中音效留空间；后续按 A3 换定制曲。</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>未入库；待制作/采购音频文件</t>
+          <t>占位正式曲：Ninja Theme by Spring Spring，OpenGameArt CC0（公共领域，可商用免署名）；OGG 原文件入库。</t>
         </is>
       </c>
     </row>
@@ -854,12 +854,12 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>res://sound/bgm/music_main_menu.ogg</t>
+          <t>res://sound/bgm/music_main_menu.wav</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>planned</t>
+          <t>imported</t>
         </is>
       </c>
       <c r="H4" s="2" t="b">
@@ -897,12 +897,12 @@
       </c>
       <c r="Q4" s="2" t="inlineStr">
         <is>
-          <t>黑暗中世纪身份主题；低弦乐、框鼓、远钟和微弱唱诗，先把世界观立住。</t>
+          <t>三国主菜单主题：宁静东方古韵（古筝/笛类音色），先立氛围；后续按 A3 音频方向换正式定制曲。</t>
         </is>
       </c>
       <c r="R4" s="2" t="inlineStr">
         <is>
-          <t>未入库；待制作/采购音频文件</t>
+          <t>占位正式曲：Oriental by Shadowfire452，OpenGameArt CC0（公共领域，可商用免署名）；WAV 原格式入库。</t>
         </is>
       </c>
     </row>

</xml_diff>